<commit_message>
Extend make_tests.py with priority-by-送出時間 and weekend-cap batches
batch-2026-11.xlsx: three rows on the same Mon-Thu window, shipped in
*reverse* 送出時間 order (row 1 latest, row 3 earliest). The verdicts
(H1 fail, H2/H3 pass) only come out right if recomputeBatch() sorts by
submittedAt before evaluating — under a broken sort that walked array
order, H1 would pass and H3 would fail.

batch-2026-12.xlsx: four bookings overlap on Sat 2026-12-12 (two via
Wed-Sat, two via Sat-Tue, so weekday slots don't compete). All four pass
under 假日上限=4; under the previous single-quota=2 the 3rd and 4th would
have failed. The 測試說明 sheet documents an optional 上限例外 walkthrough
that tightens that Saturday back to 2.

Existing batches 04-10 are also touched: the 測試說明 sheet now includes
a 送出時間 column, which was needed for the priority test and is generally
helpful when reviewing expected verdicts. The 新申請 payloads themselves
are unchanged.
</commit_message>
<xml_diff>
--- a/batch-2026-04.xlsx
+++ b/batch-2026-04.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新申請" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="測試說明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="新申請" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="測試說明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -577,6 +577,11 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>送出時間</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>預期結果</t>
         </is>
       </c>
@@ -615,6 +620,11 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>2026-04-05 09:00</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>通過</t>
         </is>
       </c>
@@ -653,6 +663,11 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>2026-04-05 10:00</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>未通過 - 超出可預約範圍</t>
         </is>
       </c>
@@ -690,6 +705,11 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-04-05 11:00</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>通過</t>
         </is>

</xml_diff>